<commit_message>
disciplinas: CT-DISC-07 a 13, Page Object e matriz atualizada
Automacao:
- disc.cy.js vai de 6 para 13 testes (CT-DISC-01 a 13)
- CT-DISC-07 e CT-DISC-13 marcados com it.skip, documentando BUG-02 e
  BUG-03: sao defeitos confirmados do sistema, nao falhas de teste, e
  ficariam vermelhos na esteira sem provar nada de novo
- novo Page Object pages/disciplinas, reaproveitando o de login
- CT-DISC-13: seletor corrigido de cy.get('tr, Matematica') para
  cy.contains('tr', 'Matematica'); a versao anterior era lista de
  seletores CSS e acertava a linha por coincidencia de ordem
- modal de confirmacao ancorado em data-testid

Documentacao:
- BUG-03 detalhado: o vinculo orfao atinge todos os professores ligados
  a disciplina excluida, nao so o criado para o teste. "Carlos Pereira",
  do cadastro inicial, passou a exibir "- Ciencias"

Suite: 32 testes, 30 passando, 2 pendentes, 0 falhando.
</commit_message>
<xml_diff>
--- a/Casos-de-Teste-EscolaNotas.xlsx
+++ b/Casos-de-Teste-EscolaNotas.xlsx
@@ -745,10 +745,10 @@
     <t xml:space="preserve">Ao excluir o registro que está em edição, o sistema deveria limpar ou fechar o formulário, impedindo a edição de algo que não existe mais.</t>
   </si>
   <si>
-    <t xml:space="preserve">O formulário permanece preenchido e com o título "Editar disciplina". Ao clicar em "Salvar", nada acontece: o sistema não exibe "Disciplina atualizada!", não exibe erro e não grava nada — a falha é silenciosa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Defeito confirmado. Ver aba Defeitos (BUG-02). Tipo alterado de Exploratório para Negativo: há falha funcional, não apenas comportamento não especificado.</t>
+    <t xml:space="preserve">O formulário permanece preenchido e com o título "Editar disciplina". Ao clicar em "Salvar", a aplicação lança a exceção "TypeError: Cannot set properties of undefined (setting 'nome')" e nada é gravado. Na tela não aparece confirmação nem mensagem de erro: para o usuário, a falha é silenciosa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defeito confirmado. Ver aba Defeitos (BUG-02). Tipo alterado de Exploratório para Negativo: há falha funcional, não apenas comportamento não especificado. Resultado obtido detalhado após execução automatizada, que expôs a exceção de JavaScript por trás da falha silenciosa.</t>
   </si>
   <si>
     <t xml:space="preserve">CT-DISC-08</t>
@@ -845,7 +845,7 @@
     <t xml:space="preserve">O sistema deveria avisar que existe professor vinculado ou impedir a exclusão, já que o RF03 exige ao menos 1 disciplina por professor.</t>
   </si>
   <si>
-    <t xml:space="preserve">A disciplina é excluída sem nenhum aviso. Na lista de Professores, "Teste A" passa a exibir um traço ("—") no lugar da disciplina, ficando sem nenhuma disciplina válida e violando a regra do próprio requisito.</t>
+    <t xml:space="preserve">A disciplina é excluída sem nenhum aviso. Na lista de Professores, "Teste A" passa a exibir um traço ("—") no lugar da disciplina, ficando sem nenhuma disciplina válida e violando a regra do próprio requisito. O efeito atinge todos os professores ligados à disciplina: "Carlos Pereira", que já vem cadastrado, passou a exibir "— Ciências".</t>
   </si>
   <si>
     <t xml:space="preserve">Defeito confirmado. Ver aba Defeitos (BUG-03). Resultado obtido detalhado após verificação: o vínculo não é removido, fica apontando para uma disciplina inexistente.</t>
@@ -1118,10 +1118,11 @@
     <t xml:space="preserve">Ao excluir o registro em edição, o formulário deveria ser limpo ou fechado.</t>
   </si>
   <si>
-    <t xml:space="preserve">O formulário continua preenchido e com o título "Editar disciplina". Ao salvar, o sistema não exibe confirmação, não exibe erro e não grava nada — falha silenciosa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O usuário acredita ter salvo uma alteração que nunca aconteceu. A ausência de qualquer retorno na tela é o que agrava a severidade.</t>
+    <t xml:space="preserve">O formulário continua preenchido e com o título "Editar disciplina". Ao salvar, a aplicação lança "TypeError: Cannot set properties of undefined (setting 'nome')" e a alteração não é gravada. A exceção não aparece para o usuário: na tela não há confirmação nem mensagem de erro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Causa raiz: ao excluir, o sistema não limpa a variável que guarda o id do registro em edição. Na hora de salvar, a busca por esse id retorna undefined e o código tenta escrever numa referência inexistente, lançando a exceção.
+Severidade Alta por ser exceção não tratada com perda silenciosa de dado: o usuário acredita ter salvo algo que nunca foi gravado. Prioridade Média porque depende de uma sequência pouco frequente (excluir o registro que está aberto em edição) e é contornável recarregando a página.</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-03</t>
@@ -1139,7 +1140,7 @@
     <t xml:space="preserve">O sistema deveria impedir a exclusão ou avisar que existe professor vinculado, já que o RF03 exige ao menos 1 disciplina por professor.</t>
   </si>
   <si>
-    <t xml:space="preserve">A exclusão acontece sem aviso. O professor passa a exibir "—" na coluna Disciplinas, ficando sem nenhuma disciplina válida.</t>
+    <t xml:space="preserve">A exclusão acontece sem aviso. O professor passa a exibir "—" na coluna Disciplinas, ficando sem nenhuma disciplina válida. Atinge todos os professores vinculados, não só o criado para o teste: "Carlos Pereira", do cadastro inicial, passou a exibir "— Ciências".</t>
   </si>
   <si>
     <t xml:space="preserve">Quebra de integridade referencial: o vínculo continua apontando para um registro que não existe mais. O sistema já faz essa limpeza para Turmas, mas não para Professores — a inconsistência sugere esquecimento na implementação.</t>
@@ -3309,7 +3310,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
         <v>219</v>
       </c>
@@ -4174,7 +4175,7 @@
       </c>
       <c r="K2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>301</v>
       </c>
@@ -4187,8 +4188,8 @@
       <c r="D3" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="E3" s="7" t="s">
-        <v>33</v>
+      <c r="E3" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>33</v>

</xml_diff>